<commit_message>
Update profils métier 2cb77cdf67d04487e6427f98c04d9e890bf41b8d
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-Responsable.xlsx
+++ b/main/ig/StructureDefinition-Responsable.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-22T14:43:59+00:00</t>
+    <t>2025-04-23T09:14:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -255,7 +255,7 @@
     <t>*</t>
   </si>
   <si>
-    <t>Responsable.dateHeureAttestationValidite</t>
+    <t>Responsable.dateHeurePriseResponsabilite</t>
   </si>
   <si>
     <t xml:space="preserve">dateTime
@@ -265,7 +265,7 @@
     <t>Date/Heure de la prise de responsabilité.</t>
   </si>
   <si>
-    <t>Responsable.Responsable</t>
+    <t>Responsable.responsable</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PersonneStructure
@@ -577,8 +577,8 @@
   <dimension ref="A1:AJ4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="34.328125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="34.328125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="35.0390625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="35.0390625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -608,7 +608,7 @@
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="34.328125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="35.0390625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>

</xml_diff>